<commit_message>
Bible added: half slide, easy navigation, verses navigation
</commit_message>
<xml_diff>
--- a/Tables.xlsx
+++ b/Tables.xlsx
@@ -1509,7 +1509,7 @@
         </is>
       </c>
       <c r="M2" s="83" t="n">
-        <v>1742</v>
+        <v>1743</v>
       </c>
       <c r="N2" s="84" t="n"/>
       <c r="R2" s="2" t="n"/>
@@ -1687,7 +1687,7 @@
         <v/>
       </c>
       <c r="F7" s="35" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G7" s="36" t="inlineStr">
         <is>
@@ -1832,14 +1832,14 @@
         </is>
       </c>
       <c r="D11" s="33" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E11" s="34">
         <f>VLOOKUP(D11, $A$2:$B$100, 2, FALSE)</f>
         <v/>
       </c>
       <c r="F11" s="35" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G11" s="36" t="inlineStr">
         <is>
@@ -1870,14 +1870,14 @@
         </is>
       </c>
       <c r="D12" s="33" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E12" s="34">
         <f>VLOOKUP(D12, $A$2:$B$100, 2, FALSE)</f>
         <v/>
       </c>
       <c r="F12" s="35" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="G12" s="36" t="inlineStr">
         <is>
@@ -1915,7 +1915,7 @@
         <v/>
       </c>
       <c r="F13" s="35" t="n">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="G13" s="36" t="inlineStr">
         <is>
@@ -2006,14 +2006,14 @@
     </row>
     <row r="16" ht="21" customHeight="1" s="53">
       <c r="D16" s="33" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E16" s="34">
         <f>VLOOKUP(D16, $A$2:$B$100, 2, FALSE)</f>
         <v/>
       </c>
       <c r="F16" s="35" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G16" s="36" t="inlineStr">
         <is>
@@ -2036,14 +2036,14 @@
     </row>
     <row r="17" ht="21.75" customHeight="1" s="53" thickBot="1">
       <c r="D17" s="33" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E17" s="34">
         <f>VLOOKUP(D17, $A$2:$B$100, 2, FALSE)</f>
         <v/>
       </c>
       <c r="F17" s="35" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="G17" s="36" t="inlineStr">
         <is>
@@ -2066,14 +2066,14 @@
     </row>
     <row r="18" ht="21.75" customHeight="1" s="53" thickTop="1">
       <c r="D18" s="33" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E18" s="34">
         <f>VLOOKUP(D18, $A$2:$B$100, 2, FALSE)</f>
         <v/>
       </c>
       <c r="F18" s="35" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="G18" s="36" t="inlineStr">
         <is>
@@ -2102,7 +2102,7 @@
         <v/>
       </c>
       <c r="F19" s="35" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="G19" s="36" t="inlineStr">
         <is>
@@ -2131,7 +2131,7 @@
         <v/>
       </c>
       <c r="F20" s="35" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="G20" s="36" t="inlineStr">
         <is>
@@ -2160,7 +2160,7 @@
         <v/>
       </c>
       <c r="F21" s="35" t="n">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="G21" s="36" t="inlineStr">
         <is>
@@ -2189,7 +2189,7 @@
         <v/>
       </c>
       <c r="F22" s="35" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="G22" s="36" t="inlineStr">
         <is>
@@ -2229,14 +2229,14 @@
     </row>
     <row r="24" ht="21" customHeight="1" s="53">
       <c r="D24" s="37" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E24" s="34">
         <f>VLOOKUP(D24, $A$2:$B$100, 2, FALSE)</f>
         <v/>
       </c>
       <c r="F24" s="38" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="G24" s="39" t="inlineStr">
         <is>
@@ -2257,14 +2257,14 @@
     </row>
     <row r="25" ht="21" customHeight="1" s="53">
       <c r="D25" s="37" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E25" s="34">
         <f>VLOOKUP(D25, $A$2:$B$100, 2, FALSE)</f>
         <v/>
       </c>
       <c r="F25" s="38" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="G25" s="39" t="inlineStr">
         <is>
@@ -2272,7 +2272,7 @@
         </is>
       </c>
       <c r="I25" s="12" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J25" s="15">
         <f>VLOOKUP(I25,I3:J21, 2, FALSE)</f>
@@ -2448,7 +2448,7 @@
     </row>
     <row r="2" ht="15.75" customHeight="1" s="53">
       <c r="A2" s="8" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="B2" s="8" t="n">
         <v>8</v>
@@ -2479,7 +2479,7 @@
     </row>
     <row r="3">
       <c r="A3" s="47" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="B3" s="47" t="n">
         <v>8</v>
@@ -2506,7 +2506,7 @@
     </row>
     <row r="4">
       <c r="A4" s="47" t="n">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="B4" s="47" t="n">
         <v>8</v>
@@ -2533,7 +2533,7 @@
     </row>
     <row r="5">
       <c r="A5" s="47" t="n">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B5" s="47" t="n">
         <v>8</v>
@@ -2560,7 +2560,7 @@
     </row>
     <row r="6">
       <c r="A6" s="47" t="n">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="B6" s="47" t="n">
         <v>8</v>
@@ -2587,7 +2587,7 @@
     </row>
     <row r="7">
       <c r="A7" s="47" t="n">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="B7" s="47" t="n">
         <v>8</v>
@@ -2614,7 +2614,7 @@
     </row>
     <row r="8">
       <c r="A8" s="47" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B8" s="47" t="n">
         <v>8</v>
@@ -2641,10 +2641,10 @@
     </row>
     <row r="9">
       <c r="A9" s="47" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="B9" s="47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C9" s="47" t="n">
         <v>161</v>
@@ -2668,10 +2668,10 @@
     </row>
     <row r="10">
       <c r="A10" s="47" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="B10" s="47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C10" s="47" t="n">
         <v>182</v>
@@ -2695,10 +2695,10 @@
     </row>
     <row r="11">
       <c r="A11" s="47" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="B11" s="47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C11" s="47" t="n">
         <v>194</v>
@@ -2722,10 +2722,10 @@
     </row>
     <row r="12">
       <c r="A12" s="47" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="B12" s="47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C12" s="47" t="n">
         <v>203</v>
@@ -2749,10 +2749,10 @@
     </row>
     <row r="13">
       <c r="A13" s="47" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="B13" s="47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C13" s="47" t="n">
         <v>214</v>
@@ -2776,10 +2776,10 @@
     </row>
     <row r="14">
       <c r="A14" s="47" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B14" s="47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C14" s="47" t="n">
         <v>225</v>
@@ -2803,10 +2803,10 @@
     </row>
     <row r="15">
       <c r="A15" s="47" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B15" s="47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C15" s="47" t="n">
         <v>233</v>
@@ -2830,10 +2830,10 @@
     </row>
     <row r="16">
       <c r="A16" s="47" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B16" s="47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C16" s="47" t="n">
         <v>247</v>
@@ -2857,10 +2857,10 @@
     </row>
     <row r="17">
       <c r="A17" s="47" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="B17" s="47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C17" s="47" t="n">
         <v>265</v>
@@ -2884,10 +2884,10 @@
     </row>
     <row r="18">
       <c r="A18" s="47" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B18" s="47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C18" s="47" t="n">
         <v>273</v>
@@ -2911,10 +2911,10 @@
     </row>
     <row r="19">
       <c r="A19" s="47" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B19" s="47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C19" s="47" t="n">
         <v>286</v>
@@ -2938,10 +2938,10 @@
     </row>
     <row r="20">
       <c r="A20" s="47" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="B20" s="47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C20" s="47" t="n">
         <v>295</v>
@@ -2965,10 +2965,10 @@
     </row>
     <row r="21">
       <c r="A21" s="47" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="B21" s="47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C21" s="47" t="n">
         <v>305</v>
@@ -2992,10 +2992,10 @@
     </row>
     <row r="22">
       <c r="A22" s="47" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="B22" s="47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C22" s="47" t="n">
         <v>317</v>
@@ -3019,10 +3019,10 @@
     </row>
     <row r="23">
       <c r="A23" s="47" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="B23" s="47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C23" s="47" t="n">
         <v>335</v>
@@ -3046,10 +3046,10 @@
     </row>
     <row r="24">
       <c r="A24" s="47" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="B24" s="47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C24" s="47" t="n">
         <v>365</v>
@@ -3073,10 +3073,10 @@
     </row>
     <row r="25">
       <c r="A25" s="47" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="B25" s="47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C25" s="47" t="n">
         <v>377</v>
@@ -3100,10 +3100,10 @@
     </row>
     <row r="26">
       <c r="A26" s="47" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="B26" s="47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C26" s="47" t="n">
         <v>385</v>
@@ -3127,10 +3127,10 @@
     </row>
     <row r="27">
       <c r="A27" s="47" t="n">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="B27" s="47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C27" s="47" t="n">
         <v>402</v>
@@ -3154,10 +3154,10 @@
     </row>
     <row r="28">
       <c r="A28" s="47" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B28" s="47" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C28" s="47" t="n">
         <v>414</v>
@@ -3181,7 +3181,7 @@
     </row>
     <row r="29">
       <c r="A29" s="47" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="B29" s="47" t="n">
         <v>9</v>
@@ -3208,7 +3208,7 @@
     </row>
     <row r="30">
       <c r="A30" s="47" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="B30" s="47" t="n">
         <v>9</v>
@@ -3235,7 +3235,7 @@
     </row>
     <row r="31">
       <c r="A31" s="47" t="n">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="B31" s="47" t="n">
         <v>9</v>
@@ -3262,7 +3262,7 @@
     </row>
     <row r="32">
       <c r="A32" s="47" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="B32" s="47" t="n">
         <v>9</v>
@@ -3289,7 +3289,7 @@
     </row>
     <row r="33">
       <c r="A33" s="47" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="B33" s="47" t="n">
         <v>9</v>
@@ -3316,7 +3316,7 @@
     </row>
     <row r="34">
       <c r="A34" s="47" t="n">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="B34" s="47" t="n">
         <v>9</v>
@@ -3343,7 +3343,7 @@
     </row>
     <row r="35">
       <c r="A35" s="47" t="n">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B35" s="47" t="n">
         <v>9</v>
@@ -3370,7 +3370,7 @@
     </row>
     <row r="36">
       <c r="A36" s="47" t="n">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="B36" s="47" t="n">
         <v>9</v>
@@ -3397,7 +3397,7 @@
     </row>
     <row r="37">
       <c r="A37" s="47" t="n">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="B37" s="47" t="n">
         <v>9</v>
@@ -3424,7 +3424,7 @@
     </row>
     <row r="38">
       <c r="A38" s="47" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B38" s="47" t="n">
         <v>9</v>
@@ -3451,10 +3451,10 @@
     </row>
     <row r="39">
       <c r="A39" s="47" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="B39" s="47" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C39" s="47" t="n">
         <v>588</v>
@@ -3478,10 +3478,10 @@
     </row>
     <row r="40">
       <c r="A40" s="47" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="B40" s="47" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C40" s="47" t="n">
         <v>601</v>
@@ -3505,10 +3505,10 @@
     </row>
     <row r="41" ht="15.75" customHeight="1" s="53">
       <c r="A41" s="8" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="B41" s="8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C41" s="8" t="n">
         <v>616</v>
@@ -3536,10 +3536,10 @@
     </row>
     <row r="42" ht="15.75" customHeight="1" s="53">
       <c r="A42" s="47" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="B42" s="47" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C42" s="47" t="n">
         <v>639</v>
@@ -3563,10 +3563,10 @@
     </row>
     <row r="43" ht="15.75" customHeight="1" s="53">
       <c r="A43" s="47" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="B43" s="47" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C43" s="47" t="n">
         <v>657</v>
@@ -3590,10 +3590,10 @@
     </row>
     <row r="44" ht="15.75" customHeight="1" s="53">
       <c r="A44" s="47" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B44" s="47" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C44" s="47" t="n">
         <v>672</v>
@@ -3617,10 +3617,10 @@
     </row>
     <row r="45" ht="15.75" customHeight="1" s="53">
       <c r="A45" s="47" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B45" s="47" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C45" s="47" t="n">
         <v>692</v>
@@ -3644,10 +3644,10 @@
     </row>
     <row r="46" ht="15.75" customHeight="1" s="53">
       <c r="A46" s="47" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B46" s="47" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C46" s="47" t="n">
         <v>708</v>
@@ -3671,10 +3671,10 @@
     </row>
     <row r="47" ht="15.75" customHeight="1" s="53">
       <c r="A47" s="47" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="B47" s="47" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C47" s="47" t="n">
         <v>721</v>
@@ -3698,10 +3698,10 @@
     </row>
     <row r="48" ht="15.75" customHeight="1" s="53">
       <c r="A48" s="47" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B48" s="47" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C48" s="47" t="n">
         <v>738</v>
@@ -3725,10 +3725,10 @@
     </row>
     <row r="49" ht="15.75" customHeight="1" s="53">
       <c r="A49" s="47" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B49" s="47" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C49" s="47" t="n">
         <v>754</v>
@@ -3752,10 +3752,10 @@
     </row>
     <row r="50" ht="15.75" customHeight="1" s="53">
       <c r="A50" s="47" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="B50" s="47" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C50" s="47" t="n">
         <v>765</v>
@@ -3779,10 +3779,10 @@
     </row>
     <row r="51" ht="15.75" customHeight="1" s="53">
       <c r="A51" s="8" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="B51" s="8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C51" s="8" t="n">
         <v>791</v>
@@ -18231,10 +18231,10 @@
     </row>
     <row r="2">
       <c r="A2" s="47" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="B2" s="47" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" s="47" t="n">
         <v>2</v>
@@ -18278,10 +18278,10 @@
     </row>
     <row r="3">
       <c r="A3" s="47" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="B3" s="47" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C3" s="47" t="inlineStr"/>
       <c r="D3" s="47" t="inlineStr"/>
@@ -18319,10 +18319,10 @@
     </row>
     <row r="4">
       <c r="A4" s="47" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="B4" s="47" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C4" s="47" t="inlineStr"/>
       <c r="D4" s="47" t="inlineStr"/>
@@ -18360,10 +18360,10 @@
     </row>
     <row r="5">
       <c r="A5" s="47" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="B5" s="47" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C5" s="47" t="inlineStr"/>
       <c r="D5" s="47" t="inlineStr"/>
@@ -18532,7 +18532,7 @@
     </row>
     <row r="2">
       <c r="A2" s="43" t="n">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B2" s="43" t="n">
         <v>6</v>
@@ -18585,7 +18585,7 @@
     </row>
     <row r="3">
       <c r="A3" s="43" t="n">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="B3" s="43" t="n">
         <v>6</v>
@@ -18644,7 +18644,7 @@
     </row>
     <row r="4">
       <c r="A4" s="43" t="n">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="B4" s="43" t="n">
         <v>6</v>
@@ -18693,7 +18693,7 @@
     </row>
     <row r="5">
       <c r="A5" s="43" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B5" s="43" t="n">
         <v>6</v>
@@ -18738,10 +18738,10 @@
     </row>
     <row r="6">
       <c r="A6" s="43" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="B6" s="43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C6" s="43" t="n"/>
       <c r="D6" s="43" t="n"/>
@@ -18783,10 +18783,10 @@
     </row>
     <row r="7">
       <c r="A7" s="43" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="B7" s="43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C7" s="43" t="n"/>
       <c r="D7" s="43" t="n"/>
@@ -18828,10 +18828,10 @@
     </row>
     <row r="8">
       <c r="A8" s="43" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="B8" s="43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C8" s="43" t="n"/>
       <c r="D8" s="43" t="n"/>
@@ -18873,10 +18873,10 @@
     </row>
     <row r="9">
       <c r="A9" s="43" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="B9" s="43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C9" s="43" t="n"/>
       <c r="D9" s="43" t="n"/>
@@ -18916,10 +18916,10 @@
     </row>
     <row r="10">
       <c r="A10" s="43" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="B10" s="43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C10" s="43" t="n">
         <v>342</v>
@@ -18975,10 +18975,10 @@
     </row>
     <row r="11">
       <c r="A11" s="43" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B11" s="43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C11" s="43" t="n"/>
       <c r="D11" s="43" t="n"/>
@@ -19020,10 +19020,10 @@
     </row>
     <row r="12">
       <c r="A12" s="43" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B12" s="43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C12" s="43" t="n"/>
       <c r="D12" s="43" t="n"/>
@@ -19065,10 +19065,10 @@
     </row>
     <row r="13">
       <c r="A13" s="43" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B13" s="43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C13" s="43" t="n"/>
       <c r="D13" s="43" t="n"/>
@@ -19110,10 +19110,10 @@
     </row>
     <row r="14">
       <c r="A14" s="43" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="B14" s="43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C14" s="43" t="n"/>
       <c r="D14" s="43" t="n"/>
@@ -19155,10 +19155,10 @@
     </row>
     <row r="15">
       <c r="A15" s="43" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B15" s="43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C15" s="43" t="n"/>
       <c r="D15" s="43" t="n"/>
@@ -19200,10 +19200,10 @@
     </row>
     <row r="16">
       <c r="A16" s="43" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B16" s="43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C16" s="43" t="n"/>
       <c r="D16" s="43" t="n"/>
@@ -19243,10 +19243,10 @@
     </row>
     <row r="17">
       <c r="A17" s="43" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="B17" s="43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C17" s="43" t="n">
         <v>658</v>
@@ -19302,10 +19302,10 @@
     </row>
     <row r="18">
       <c r="A18" s="43" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="B18" s="43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C18" s="43" t="n"/>
       <c r="D18" s="43" t="n"/>
@@ -19347,10 +19347,10 @@
     </row>
     <row r="19">
       <c r="A19" s="43" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="B19" s="43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C19" s="43" t="n"/>
       <c r="D19" s="43" t="n"/>
@@ -19392,10 +19392,10 @@
     </row>
     <row r="20">
       <c r="A20" s="43" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="B20" s="43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C20" s="43" t="n"/>
       <c r="D20" s="43" t="n"/>
@@ -19437,10 +19437,10 @@
     </row>
     <row r="21">
       <c r="A21" s="43" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="B21" s="43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C21" s="43" t="n"/>
       <c r="D21" s="43" t="n"/>
@@ -19482,10 +19482,10 @@
     </row>
     <row r="22">
       <c r="A22" s="43" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="B22" s="43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C22" s="43" t="n"/>
       <c r="D22" s="43" t="n"/>
@@ -19527,10 +19527,10 @@
     </row>
     <row r="23">
       <c r="A23" s="43" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="B23" s="43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C23" s="43" t="n"/>
       <c r="D23" s="43" t="n"/>
@@ -19570,10 +19570,10 @@
     </row>
     <row r="24">
       <c r="A24" s="43" t="n">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="B24" s="43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C24" s="43" t="n">
         <v>1059</v>
@@ -19629,10 +19629,10 @@
     </row>
     <row r="25">
       <c r="A25" s="43" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B25" s="43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C25" s="43" t="n"/>
       <c r="D25" s="43" t="n"/>
@@ -19674,7 +19674,7 @@
     </row>
     <row r="26">
       <c r="A26" s="43" t="n">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="B26" s="43" t="n">
         <v>7</v>
@@ -19719,7 +19719,7 @@
     </row>
     <row r="27">
       <c r="A27" s="43" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="B27" s="43" t="n">
         <v>7</v>
@@ -19764,7 +19764,7 @@
     </row>
     <row r="28">
       <c r="A28" s="43" t="n">
-        <v>3</v>
+        <v>23</v>
       </c>
       <c r="B28" s="43" t="n">
         <v>7</v>
@@ -19809,7 +19809,7 @@
     </row>
     <row r="29">
       <c r="A29" s="43" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="B29" s="43" t="n">
         <v>7</v>
@@ -19854,7 +19854,7 @@
     </row>
     <row r="30">
       <c r="A30" s="43" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="B30" s="43" t="n">
         <v>7</v>
@@ -19897,7 +19897,7 @@
     </row>
     <row r="31">
       <c r="A31" s="43" t="n">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="B31" s="43" t="n">
         <v>7</v>
@@ -19956,7 +19956,7 @@
     </row>
     <row r="32">
       <c r="A32" s="43" t="n">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B32" s="43" t="n">
         <v>7</v>
@@ -20001,7 +20001,7 @@
     </row>
     <row r="33">
       <c r="A33" s="43" t="n">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="B33" s="43" t="n">
         <v>7</v>
@@ -20046,7 +20046,7 @@
     </row>
     <row r="34">
       <c r="A34" s="43" t="n">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="B34" s="43" t="n">
         <v>7</v>
@@ -20091,7 +20091,7 @@
     </row>
     <row r="35">
       <c r="A35" s="43" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B35" s="43" t="n">
         <v>7</v>
@@ -20136,10 +20136,10 @@
     </row>
     <row r="36">
       <c r="A36" s="43" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="B36" s="43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C36" s="43" t="n"/>
       <c r="D36" s="43" t="n"/>
@@ -20181,10 +20181,10 @@
     </row>
     <row r="37">
       <c r="A37" s="43" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="B37" s="43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C37" s="43" t="n"/>
       <c r="D37" s="43" t="n"/>
@@ -20224,10 +20224,10 @@
     </row>
     <row r="38">
       <c r="A38" s="43" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="B38" s="43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C38" s="43" t="n">
         <v>2023</v>
@@ -20283,10 +20283,10 @@
     </row>
     <row r="39">
       <c r="A39" s="43" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="B39" s="43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C39" s="43" t="n"/>
       <c r="D39" s="43" t="n"/>
@@ -20328,10 +20328,10 @@
     </row>
     <row r="40">
       <c r="A40" s="43" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="B40" s="43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C40" s="43" t="n"/>
       <c r="D40" s="43" t="n"/>
@@ -20373,10 +20373,10 @@
     </row>
     <row r="41">
       <c r="A41" s="43" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B41" s="43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C41" s="43" t="n"/>
       <c r="D41" s="43" t="n"/>
@@ -20418,10 +20418,10 @@
     </row>
     <row r="42">
       <c r="A42" s="43" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B42" s="43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C42" s="43" t="n"/>
       <c r="D42" s="43" t="n"/>
@@ -20463,10 +20463,10 @@
     </row>
     <row r="43">
       <c r="A43" s="43" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B43" s="43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C43" s="43" t="n"/>
       <c r="D43" s="43" t="n"/>
@@ -20508,10 +20508,10 @@
     </row>
     <row r="44">
       <c r="A44" s="43" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="B44" s="43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C44" s="43" t="n"/>
       <c r="D44" s="43" t="n"/>
@@ -20551,10 +20551,10 @@
     </row>
     <row r="45">
       <c r="A45" s="43" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B45" s="43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C45" s="43" t="n">
         <v>2619</v>
@@ -20610,10 +20610,10 @@
     </row>
     <row r="46">
       <c r="A46" s="43" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B46" s="43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C46" s="43" t="n"/>
       <c r="D46" s="43" t="n"/>
@@ -20655,10 +20655,10 @@
     </row>
     <row r="47">
       <c r="A47" s="43" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="B47" s="43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C47" s="43" t="n"/>
       <c r="D47" s="43" t="n"/>
@@ -20700,10 +20700,10 @@
     </row>
     <row r="48">
       <c r="A48" s="43" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="B48" s="43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C48" s="43" t="n"/>
       <c r="D48" s="43" t="n"/>
@@ -20745,10 +20745,10 @@
     </row>
     <row r="49">
       <c r="A49" s="43" t="n">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="B49" s="43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C49" s="43" t="n"/>
       <c r="D49" s="43" t="n"/>
@@ -20790,10 +20790,10 @@
     </row>
     <row r="50">
       <c r="A50" s="43" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="B50" s="43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C50" s="43" t="n"/>
       <c r="D50" s="43" t="n"/>
@@ -20835,10 +20835,10 @@
     </row>
     <row r="51">
       <c r="A51" s="43" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="B51" s="43" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C51" s="43" t="n"/>
       <c r="D51" s="43" t="n"/>
@@ -21029,10 +21029,10 @@
     </row>
     <row r="2" ht="23.25" customHeight="1" s="53">
       <c r="A2" s="46" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="B2" s="46" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" s="46" t="n">
         <v>1</v>

</xml_diff>